<commit_message>
Updated event names from Events.xlsx
</commit_message>
<xml_diff>
--- a/Events.xlsx
+++ b/Events.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/harryscons/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/harryscons/Documents/Antigravity/RaceSystem/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9888F660-D5CC-1E40-B0ED-5D338814AC0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ABD4A0B3-D68B-D647-90A4-FBB4FC1200BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="11980" yWindow="5980" windowWidth="27640" windowHeight="16680" xr2:uid="{F7D071DF-A808-7747-8BAE-A2EB7F114212}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
   <si>
     <t>100μ</t>
   </si>
@@ -54,9 +54,6 @@
   </si>
   <si>
     <t>1500μ</t>
-  </si>
-  <si>
-    <t>3000μ</t>
   </si>
   <si>
     <t>5000μ</t>
@@ -480,7 +477,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6DD016C4-6F37-7249-8B9D-C66FA84C8C79}">
-  <dimension ref="A1:A21"/>
+  <dimension ref="A1:A20"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.2">
@@ -583,11 +580,6 @@
         <v>19</v>
       </c>
     </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A21" s="1" t="s">
-        <v>20</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>